<commit_message>
Fix in Config, Filepaths deleted and transfered into Orchestratorassets
</commit_message>
<xml_diff>
--- a/Medavis Webex Report/Data/Config.xlsx
+++ b/Medavis Webex Report/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicolas.jahl\develop\uipath\uipath-rpa_med\Medavis Webex Report\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E59CB859-A8C8-4F76-978C-8EADF04DA68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47FBD29B-80A1-4426-877B-4B8AE8FE7F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="72">
   <si>
     <t>Name</t>
   </si>
@@ -217,12 +217,6 @@
     <t>Utility path for saving temporary files. If left empty or not rooted a default folder is set . Will be deleted at end.</t>
   </si>
   <si>
-    <t>CriteriaListPath</t>
-  </si>
-  <si>
-    <t>\\fsitm\itm-ablage\Allgemein\RPA_medavis_TEST\Input\Kriterienliste_medavis-automation.gsr.xlsx</t>
-  </si>
-  <si>
     <t>EingabeFB_Zusätzliche freieTage</t>
   </si>
   <si>
@@ -232,12 +226,6 @@
     <t>C5</t>
   </si>
   <si>
-    <t>DatabaseFilePath</t>
-  </si>
-  <si>
-    <t>\\fsitm\itm-ablage\Allgemein\RPA_medavis_TEST\Datenbank\Datenbank.xlsx</t>
-  </si>
-  <si>
     <t>DatabaseFileSheet</t>
   </si>
   <si>
@@ -256,9 +244,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>WebexRoomID</t>
-  </si>
-  <si>
     <t>WebexApiUrl</t>
   </si>
   <si>
@@ -266,9 +251,6 @@
   </si>
   <si>
     <t>CriteriaListDateCell</t>
-  </si>
-  <si>
-    <t>5bb39900-29cc-11f1-a361-a1e4ed76f7fa</t>
   </si>
 </sst>
 </file>
@@ -331,7 +313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -342,12 +324,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -706,17 +686,17 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
         <v>60</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>61</v>
       </c>
       <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:26" ht="14.4">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
         <v>62</v>
@@ -725,7 +705,7 @@
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
         <v>64</v>
@@ -735,7 +715,7 @@
       <c r="A5" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" t="s">
         <v>66</v>
       </c>
       <c r="C5" s="4"/>
@@ -756,30 +736,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B10" t="s">
-        <v>75</v>
-      </c>
-    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3074,60 +3033,60 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" s="9"/>
-      <c r="B13" s="7"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="6"/>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>

</xml_diff>